<commit_message>
add dairy milk solids source data
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v01.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A249807-E525-4A13-904D-1CE9B8BAE0CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966F1FBF-890E-449E-B26D-5B7FFA1B4B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="15" windowWidth="37350" windowHeight="19740" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="780" yWindow="300" windowWidth="37350" windowHeight="19740" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -331,6 +331,12 @@
     <definedName name="SourceData_Dairy.SourceData_Dairy_EmissionFactorForLeachingAndRunoff_Unit">_xlfn.LAMBDA("kg N2O-N/kg N")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_EmissionFactorForLeachingAndRunoff_Variable">_xlfn.LAMBDA("EF_leach")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_EmissionFactorForLeachingAndRunoff_Variation">_xlfn.LAMBDA("")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Data">_xlfn.LAMBDA(4)</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Source">_xlfn.LAMBDA("VEERG 2026: 3.3.2.2 DATA (METHOD 1 AND 2 OPTIONS)")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Title">_xlfn.LAMBDA("Fat content in fat and protein corrected milk")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Unit">_xlfn.LAMBDA("percent")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Variable">_xlfn.LAMBDA("FC_j")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Variation">_xlfn.LAMBDA("")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FracGASMSoil_Data">_xlfn.LAMBDA(0.21)</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FracGASMSoil_Source">_xlfn.LAMBDA("VEERG 2026: 4.3.2.3 CONSTANTS")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_FracGASMSoil_Title">_xlfn.LAMBDA("Fraction of nitrogen volatilized from urine and faeces deposited on pasture")</definedName>
@@ -415,6 +421,12 @@
     <definedName name="SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Unit">_xlfn.LAMBDA("kg/day")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Variable">_xlfn.LAMBDA("VSj=3,5; NPWj=3,5")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_PreWeanedCalves_Variation">_xlfn.LAMBDA("VARIATION OF SOURCE: Added 'Animal class j' column header")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Data">_xlfn.LAMBDA(3.3)</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Source">_xlfn.LAMBDA("VEERG 2026: 3.3.2.2 DATA (METHOD 1 AND 2 OPTIONS)")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Title">_xlfn.LAMBDA("Protein content in fat and protein corrected milk")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Unit">_xlfn.LAMBDA("percent")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Variable">_xlfn.LAMBDA("PC_j")</definedName>
+    <definedName name="SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Variation">_xlfn.LAMBDA("")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_ReferenceWeights_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 5, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Milking Cows","Heifers &gt;1","Heifers &lt;1 (weaned)","Bulls &gt;1","Bulls &lt;1 (weaned)";590,590,590,770,770}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_ReferenceWeights_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.3.4")</definedName>
     <definedName name="SourceData_Dairy.SourceData_Dairy_ReferenceWeights_Title">_xlfn.LAMBDA("Table A.1.3.4: Dairy cattle - Reference weights (kg) (WRj)")</definedName>
@@ -5963,6 +5975,7 @@
               <a:latin typeface="Times New Roman"/>
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>Daily production of enteric methane</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="1000" b="1">
@@ -6163,6 +6176,7 @@
               <a:latin typeface="Times New Roman"/>
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
+            <a:pPr algn="ctr"/>
             <a:t>Total annual methane production from enteric fermentation in dairy cattle</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="1000" b="1">
@@ -6543,8 +6557,8 @@
       <xdr:rowOff>52387</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="4845044" cy="234103"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -6843,7 +6857,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -6908,8 +6922,8 @@
       <xdr:rowOff>214312</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1461105" cy="370551"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="TextBox 10">
@@ -7114,7 +7128,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="TextBox 10">
@@ -7392,8 +7406,8 @@
       <xdr:rowOff>125505</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1353126" cy="186333"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -7435,6 +7449,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -7536,7 +7551,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="TextBox 1">
@@ -7600,8 +7615,8 @@
       <xdr:rowOff>162728</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="7606378" cy="332079"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -7643,6 +7658,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -8137,7 +8153,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="TextBox 2">
@@ -8201,8 +8217,8 @@
       <xdr:rowOff>211708</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="8183202" cy="332079"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -8244,6 +8260,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -8756,7 +8773,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -8841,8 +8858,8 @@
       <xdr:rowOff>228600</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1606465" cy="383888"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -8884,6 +8901,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -9064,7 +9082,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -10278,7 +10296,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="650" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="856" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -14910,9 +14928,11 @@
         <v>268</v>
       </c>
       <c r="E55" s="130">
+        <f>'Constants - Dairy'!$D$221/100</f>
         <v>0.04</v>
       </c>
       <c r="F55" s="149">
+        <f>'Constants - Dairy'!$D$221/100</f>
         <v>0.04</v>
       </c>
       <c r="G55" s="2" t="s">
@@ -14925,9 +14945,11 @@
         <v>269</v>
       </c>
       <c r="E56" s="130">
+        <f>'Constants - Dairy'!$D$227/100</f>
         <v>3.3000000000000002E-2</v>
       </c>
       <c r="F56" s="149">
+        <f>'Constants - Dairy'!$D$227/100</f>
         <v>3.3000000000000002E-2</v>
       </c>
       <c r="G56" s="2" t="s">
@@ -16123,7 +16145,7 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <dataValidations disablePrompts="1" count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E109" xr:uid="{AF94BFC8-A9BD-4286-932B-111409BF1EB6}">
       <formula1>INDIRECT("Table_SourceData_Dairy_CropProdSystems[Production system]")</formula1>
     </dataValidation>
@@ -20917,76 +20939,116 @@
     <row r="216" spans="1:13" x14ac:dyDescent="0.25">
       <c r="M216" s="24"/>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="D217" s="6" t="str" cm="1">
+        <f t="array" ref="D217">SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Title()</f>
+        <v>Fat content in fat and protein corrected milk</v>
+      </c>
       <c r="M217" s="24"/>
     </row>
     <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D218" s="5" t="str" cm="1">
+        <f t="array" ref="D218">SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Source()</f>
+        <v>VEERG 2026: 3.3.2.2 DATA (METHOD 1 AND 2 OPTIONS)</v>
+      </c>
       <c r="M218" s="24"/>
     </row>
     <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D219" s="1" t="str" cm="1">
+        <f t="array" ref="D219">SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Variable()</f>
+        <v>FC_j</v>
+      </c>
       <c r="M219" s="24"/>
     </row>
     <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D220" s="57" t="str" cm="1">
+        <f t="array" ref="D220">SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Unit()</f>
+        <v>percent</v>
+      </c>
       <c r="M220" s="24"/>
     </row>
     <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D221" s="56" cm="1">
+        <f t="array" ref="D221">SourceData_Dairy.SourceData_Dairy_FatContentInMilk_Data()</f>
+        <v>4</v>
+      </c>
       <c r="M221" s="24"/>
     </row>
     <row r="222" spans="1:13" x14ac:dyDescent="0.25">
       <c r="M222" s="24"/>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="D223" s="6" t="str" cm="1">
+        <f t="array" ref="D223">SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Title()</f>
+        <v>Protein content in fat and protein corrected milk</v>
+      </c>
       <c r="M223" s="24"/>
     </row>
     <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D224" s="5" t="str" cm="1">
+        <f t="array" ref="D224">SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Source()</f>
+        <v>VEERG 2026: 3.3.2.2 DATA (METHOD 1 AND 2 OPTIONS)</v>
+      </c>
       <c r="M224" s="24"/>
     </row>
-    <row r="225" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="225" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D225" s="1" t="str" cm="1">
+        <f t="array" ref="D225">SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Variable()</f>
+        <v>PC_j</v>
+      </c>
       <c r="M225" s="24"/>
     </row>
-    <row r="226" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="226" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D226" s="57" t="str" cm="1">
+        <f t="array" ref="D226">SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Unit()</f>
+        <v>percent</v>
+      </c>
       <c r="M226" s="24"/>
     </row>
-    <row r="227" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="227" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D227" s="56" cm="1">
+        <f t="array" ref="D227">SourceData_Dairy.SourceData_Dairy_ProteinContentInMilk_Data()</f>
+        <v>3.3</v>
+      </c>
       <c r="M227" s="24"/>
     </row>
-    <row r="228" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="228" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M228" s="24"/>
     </row>
-    <row r="229" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="229" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M229" s="24"/>
     </row>
-    <row r="230" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="230" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M230" s="24"/>
     </row>
-    <row r="231" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="231" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M231" s="24"/>
     </row>
-    <row r="232" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="232" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M232" s="24"/>
     </row>
-    <row r="233" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="233" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M233" s="24"/>
     </row>
-    <row r="234" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="234" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M234" s="24"/>
     </row>
-    <row r="235" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="235" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M235" s="24"/>
     </row>
-    <row r="236" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="236" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M236" s="24"/>
     </row>
-    <row r="237" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="237" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M237" s="24"/>
     </row>
-    <row r="238" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="238" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M238" s="24"/>
     </row>
-    <row r="239" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="239" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M239" s="24"/>
     </row>
-    <row r="240" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="240" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M240" s="24"/>
     </row>
     <row r="241" spans="13:13" x14ac:dyDescent="0.25">
@@ -25765,15 +25827,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -25784,8 +25837,17 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAJwBSAGUAZgBlAHIAZQBuAGMAZQAnACwAIABhAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAGkAcwAgAGMAbwBuAHMAaQBzAHQAZQBuAHQAbAB5ACAAJwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdACcAIABhAG4AZAAgAGkAcwAgAG4AbwB0ACAAdQBzAGUAZAAgAGkAbgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAYgByAGUAZQBkAHMAXAAiACwAIAA2ADAAMAAsACAAMgAyADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAFcARwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAA1ADkAMAAsACAANQA5ADAALAAgADUAOQAwACwAIAA3ADcAMAAsACAANwA3ADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAHQAYQAgAGYAbwByACAAcAByAGUAIAAtACAAdwBlAGEAbgBlAGQAIABjAGEAbAB2AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAGoAPQAzACwANQA7ACAATgBQAFcAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagAnACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzADwAMQBcACIALAAgADAALgAwADEANwA2ACwAIAAwAC4AMgA2ADgANQAsACAAMAAuADAAMQAzADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzADwAMQBcACIALAAgADAALgAwADIAMAA0ACwAIAAwAC4AMwAwADAAMwAsACAAMAAuADAAMAA5ADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMQAwACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBOAFMAVwBcACIALAAgAFwAIgBOAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIAUwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAFYASQBDAFwAIgAsACAAXAAiAFcAQQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwAC4ANwAyACwAIAAwAC4ANwA2ACwAIAAwAC4AOAAsACAAMAAuADcAOAAsACAAMAAuADcANAAsACAAMAAuADYAOQAsACAAMAAuADcAMwAsACAAMAAuADcANgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AcwBcACIALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBzACAAKABhACkAXAAiACwAIAAwAC4AMQA1ACwAIAAwAC4AMQA4ACwAIAAwAC4ANQAwACwAIAAwAC4AMgA0ACwAIAAwAC4AMQA3ACwAIAAwAC4AMQAzACwAIAAwAC4AMQA3ACwAIAAwAC4AMQA4ACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQA7ACAARgByAGEAYwBHAEEAUwBNAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMQA3ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMgAwADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUgBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABNAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFIAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBSAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzACwAIABhAG4AZAAgAGgAbwB1AHMAZQAgAGMAbwB3AHMAXAAiACwAIAAxAC4AMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAG8AdABoAGUAcgAgAGMAYQB0AHQAbABlACAAYwBsAGEAcwBzAGUAcwBcACIALAAgADEALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABFAHgAYwBsAHUAZABlAGQAIAAnAEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQAnACAAcgBvAHcAIABhAHMAIAB0AGgAaQBzACAAaQBuAGYAbwByAG0AYQB0AGkAbwBuACAAaQBzACAAaQBuACAAdABoAGUAIAB0AGEAYgBsAGUAIAB0AGkAdABsAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHIAZQBhAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAFMAaABlAGQAXAAiACwAIABcACIARgBlAGUAZABwAGEAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAxADoAIABHAHIAYQB6AGUAZAAgAE8AbgBsAHkAXAAiACwAIAAwAC4AOAA5ACwAIAAwAC4AMQAxACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMgA6ACAATwBuACAAZgBlAGUAZABwAGEAZAAgAGYAbwByACAAPAAxADAAIABoAHIALwBkAGEAeQAgAGYAbwByACAAPAAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxACAAQQBuAGUAcgBvAGIAaQBjACAATABhAGcAbwBvAG4AXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAXAAiACwAIAAwACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADMAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAXAAiACwAIAAwACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0ANAAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABhAHkAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBvAG4AdgBlAHIAdABlAGQAIABmAHIAZQBlACAAdABlAHgAdAAgAGkAbgAgAGQAbwBjAHUAbQBlAG4AdAAgAHQAbwAgAHQAYQBiAGwAZQAsACAAbQBhAHQAYwBoAGkAbgBnACAAbABpAHYAZQBzAHQAbwBjAGsAIABjAGwAYQBzAHMAIABuAGEAbQBlAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKABwAHIAZQAtAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAXwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBEAFAAVwAnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABhACAAcwBlAHAAYQByAGEAdABlACAAaABhAG4AZABsAGkAbgBnACAAbwBmACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGQAdQByAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALABcAG4AIAAgACAAIAAyADAALgA3ACAAKgAgAEkAXwBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGEAcgBtAGwAZQB5ACAAZQB0ACAAYQBsAC4AIAAoADIAMAAxADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcAG4AVwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAXABuAEwAVwBHAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE0AUgBfAGoAIAA9ACAAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAE0ASQBfAGoAIAA9ACAAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVwBfAGoALAAgAEwAVwBHAF8AagAsACAATQBSAF8AagAsACAATQBJAF8AagAsAFwAbgAgACAAIAAgACgAMQAuADEAOAA1ACAAKwAgADAALgAwADAANAA1ADQAIAAqACAAVwBfAGoAIAAtACAAMAAuADAAMAAwADAAMAAyADYAIAAqACAAVwBfAGoAIABeACAAMgAgACsAIAAwAC4AMwAxADUAIAAqACAATABXAEcAXwBqACkAIABeACAAMgAgACoAIABNAFIAXwBqACAAKwAgAE0ASQBfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBrAGcAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAFcARwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBSAF8AagBcACIALAAgAFwAIgBpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ASQBfAGoAXAAiACwAIABcACIAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBNAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAE0ASQBfAGoAPQAoAE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQApAC8AKABHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagApAFwAbgBNAFAAXwBqACAAPQAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABMAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE4ARQAgAD0AIABuAGUAdAAgAGUAbgBlAHIAZwB5ACAAKABNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawApAFwAbgBHAEUAQwAgAD0AIABnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIAAoAE0ASgAvAGsAZwBEAE0AKQBcAG4AawAgAD0AIABlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4AcQBtAF8AagAgAD0AIABtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBQAF8AagAsACAATgBFACwAIABHAEUAQwAsACAAawAsACAAcQBtAF8AagAsAFwAbgAgACAAIAAgACgATQBQAF8AagAgACoAIAAxAC4AMAAzACAAKgAgAE4ARQApACAALwAgACgARwBFAEMAIAAqACAAawAgACoAIABxAG0AXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagA9AFwAXABmAHIAYQBjAHsATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFAH0AewBHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBcACIALAAgAFwAIgBuAGUAdAAgAGUAbgBlAHIAZwB5AFwAIgAsACAAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBFAEMAXAAiACwAIABcACIAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0AFwAIgAsACAAXAAiAE0ASgAvAGsAZwBEAE0AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBrAFwAIgAsACAAXAAiAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBtAF8AagBcACIALAAgAFwAIgBtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADYAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4ATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXABuAE0AUABfAGoAXABuAEwALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AUABfAGoAPQBNAFMAXwBqAC8AKAAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAKQBcAG4ATQBTAF8AagAgAD0AIABkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAKABrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgBDAF8AagAgAD0AIABmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAFAAQwBfAGoAIAA9ACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBTAF8AagAsACAARgBDAF8AagAsACAAUABDAF8AagAsAFwAbgAgACAAIAAgAE0AUwBfAGoAIAAvACAAKAAwAC4AMAAxACAAKgAgACgARgBDAF8AagAgACsAIABQAEMAXwBqACkAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAPQBcAFwAZgByAGEAYwB7AE0AUwBfAGoAfQB7ADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgAgAEMAbwBuAHYAZQByAHQAZQBkACAAaQBuAHAAdQB0ACAARgBDACAAYQBuAGQAIABQAEMAIABwAGUAcgBjAGUAbgB0ACAAdABvACAAaQBuAHQAZQBnAGUAcgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAbgBxAG0AXwBqAFwAbgBmAHIAYQBjAHQAaQBvAG4AXABuAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4ANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAATQBNAFMARgByAGEAYwB0AGkAbwBuACwAIABGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgATQBNAFMARgByAGEAYwB0AGkAbwBuAC0AKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4AKgBGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQAKQApAFwAbgApADsAXABuAFwAbgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACwAXABuACAAIAAgACAATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAJwBSAGUAZgBlAHIAZQBuAGMAZQAnACwAIABhAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAGkAcwAgAGMAbwBuAHMAaQBzAHQAZQBuAHQAbAB5ACAAJwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdACcAIABhAG4AZAAgAGkAcwAgAG4AbwB0ACAAdQBzAGUAZAAgAGkAbgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAYgByAGUAZQBkAHMAXAAiACwAIAA2ADAAMAAsACAAMgAyADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAFcARwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAA1ADkAMAAsACAANQA5ADAALAAgADUAOQAwACwAIAA3ADcAMAAsACAANwA3ADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAHQAYQAgAGYAbwByACAAcAByAGUAIAAtACAAdwBlAGEAbgBlAGQAIABjAGEAbAB2AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAGoAPQAzACwANQA7ACAATgBQAFcAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagAnACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzADwAMQBcACIALAAgADAALgAwADEANwA2ACwAIAAwAC4AMgA2ADgANQAsACAAMAAuADAAMQAzADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzADwAMQBcACIALAAgADAALgAwADIAMAA0ACwAIAAwAC4AMwAwADAAMwAsACAAMAAuADAAMAA5ADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMQAwACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBOAFMAVwBcACIALAAgAFwAIgBOAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIAUwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAFYASQBDAFwAIgAsACAAXAAiAFcAQQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwAC4ANwAyACwAIAAwAC4ANwA2ACwAIAAwAC4AOAAsACAAMAAuADcAOAAsACAAMAAuADcANAAsACAAMAAuADYAOQAsACAAMAAuADcAMwAsACAAMAAuADcANgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AcwBcACIALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBzACAAKABhACkAXAAiACwAIAAwAC4AMQA1ACwAIAAwAC4AMQA4ACwAIAAwAC4ANQAwACwAIAAwAC4AMgA0ACwAIAAwAC4AMQA3ACwAIAAwAC4AMQAzACwAIAAwAC4AMQA3ACwAIAAwAC4AMQA4ACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQA7ACAARgByAGEAYwBHAEEAUwBNAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMQA3ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMgAwADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUgBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABNAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFIAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBSAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzACwAIABhAG4AZAAgAGgAbwB1AHMAZQAgAGMAbwB3AHMAXAAiACwAIAAxAC4AMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAG8AdABoAGUAcgAgAGMAYQB0AHQAbABlACAAYwBsAGEAcwBzAGUAcwBcACIALAAgADEALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABFAHgAYwBsAHUAZABlAGQAIAAnAEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQAnACAAcgBvAHcAIABhAHMAIAB0AGgAaQBzACAAaQBuAGYAbwByAG0AYQB0AGkAbwBuACAAaQBzACAAaQBuACAAdABoAGUAIAB0AGEAYgBsAGUAIAB0AGkAdABsAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHIAZQBhAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAFMAaABlAGQAXAAiACwAIABcACIARgBlAGUAZABwAGEAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAxADoAIABHAHIAYQB6AGUAZAAgAE8AbgBsAHkAXAAiACwAIAAwAC4AOAA5ACwAIAAwAC4AMQAxACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMgA6ACAATwBuACAAZgBlAGUAZABwAGEAZAAgAGYAbwByACAAPAAxADAAIABoAHIALwBkAGEAeQAgAGYAbwByACAAPAAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxACAAQQBuAGUAcgBvAGIAaQBjACAATABhAGcAbwBvAG4AXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAXAAiACwAIAAwACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADMAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAXAAiACwAIAAwACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0ANAAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABhAHkAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBvAG4AdgBlAHIAdABlAGQAIABmAHIAZQBlACAAdABlAHgAdAAgAGkAbgAgAGQAbwBjAHUAbQBlAG4AdAAgAHQAbwAgAHQAYQBiAGwAZQAsACAAbQBhAHQAYwBoAGkAbgBnACAAbABpAHYAZQBzAHQAbwBjAGsAIABjAGwAYQBzAHMAIABuAGEAbQBlAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKABwAHIAZQAtAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAXwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBEAFAAVwAnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABhACAAcwBlAHAAYQByAGEAdABlACAAaABhAG4AZABsAGkAbgBnACAAbwBmACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGQAdQByAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALABcAG4AIAAgACAAIAAyADAALgA3ACAAKgAgAEkAXwBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGEAcgBtAGwAZQB5ACAAZQB0ACAAYQBsAC4AIAAoADIAMAAxADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcAG4AVwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAXABuAEwAVwBHAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE0AUgBfAGoAIAA9ACAAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAE0ASQBfAGoAIAA9ACAAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVwBfAGoALAAgAEwAVwBHAF8AagAsACAATQBSAF8AagAsACAATQBJAF8AagAsAFwAbgAgACAAIAAgACgAMQAuADEAOAA1ACAAKwAgADAALgAwADAANAA1ADQAIAAqACAAVwBfAGoAIAAtACAAMAAuADAAMAAwADAAMAAyADYAIAAqACAAVwBfAGoAIABeACAAMgAgACsAIAAwAC4AMwAxADUAIAAqACAATABXAEcAXwBqACkAIABeACAAMgAgACoAIABNAFIAXwBqACAAKwAgAE0ASQBfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBrAGcAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAFcARwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBSAF8AagBcACIALAAgAFwAIgBpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ASQBfAGoAXAAiACwAIABcACIAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBNAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAE0ASQBfAGoAPQAoAE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQApAC8AKABHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagApAFwAbgBNAFAAXwBqACAAPQAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABMAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE4ARQAgAD0AIABuAGUAdAAgAGUAbgBlAHIAZwB5ACAAKABNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawApAFwAbgBHAEUAQwAgAD0AIABnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIAAoAE0ASgAvAGsAZwBEAE0AKQBcAG4AawAgAD0AIABlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4AcQBtAF8AagAgAD0AIABtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBQAF8AagAsACAATgBFACwAIABHAEUAQwAsACAAawAsACAAcQBtAF8AagAsAFwAbgAgACAAIAAgACgATQBQAF8AagAgACoAIAAxAC4AMAAzACAAKgAgAE4ARQApACAALwAgACgARwBFAEMAIAAqACAAawAgACoAIABxAG0AXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagA9AFwAXABmAHIAYQBjAHsATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFAH0AewBHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBcACIALAAgAFwAIgBuAGUAdAAgAGUAbgBlAHIAZwB5AFwAIgAsACAAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBFAEMAXAAiACwAIABcACIAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0AFwAIgAsACAAXAAiAE0ASgAvAGsAZwBEAE0AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBrAFwAIgAsACAAXAAiAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBtAF8AagBcACIALAAgAFwAIgBtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADYAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4ATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXABuAE0AUABfAGoAXABuAEwALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AUABfAGoAPQBNAFMAXwBqAC8AKAAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAKQBcAG4ATQBTAF8AagAgAD0AIABkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAKABrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgBDAF8AagAgAD0AIABmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAFAAQwBfAGoAIAA9ACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBTAF8AagAsACAARgBDAF8AagAsACAAUABDAF8AagAsAFwAbgAgACAAIAAgAE0AUwBfAGoAIAAvACAAKAAwAC4AMAAxACAAKgAgACgARgBDAF8AagAgACsAIABQAEMAXwBqACkAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAPQBcAFwAZgByAGEAYwB7AE0AUwBfAGoAfQB7ADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgAgAEMAbwBuAHYAZQByAHQAZQBkACAAaQBuAHAAdQB0ACAARgBDACAAYQBuAGQAIABQAEMAIABwAGUAcgBjAGUAbgB0ACAAdABvACAAaQBuAHQAZQBnAGUAcgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAbgBxAG0AXwBqAFwAbgBmAHIAYQBjAHQAaQBvAG4AXABuAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4ANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAATQBNAFMARgByAGEAYwB0AGkAbwBuACwAIABGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgATQBNAFMARgByAGEAYwB0AGkAbwBuAC0AKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4AKgBGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQAKQApAFwAbgApADsAXABuAFwAbgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACwAXABuACAAIAAgACAATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25808,20 +25870,20 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
     <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
fix qm decimal place error
</commit_message>
<xml_diff>
--- a/Excel/3_3_Enteric_Dairy_WIP_v01.xlsx
+++ b/Excel/3_3_Enteric_Dairy_WIP_v01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{966F1FBF-890E-449E-B26D-5B7FFA1B4B58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8339E3F6-CC41-4756-BD54-D443D93A7722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="300" windowWidth="37350" windowHeight="19740" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="435" yWindow="30" windowWidth="37920" windowHeight="20415" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -24,9 +24,6 @@
     <sheet name="Constants - Livestock" sheetId="43" r:id="rId9"/>
     <sheet name="Acknowledgements" sheetId="72" r:id="rId10"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId11"/>
-  </externalReferences>
   <definedNames>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e">_xlfn.LAMBDA(_xlpm.E_CH4,_xlpm.GWP_CH4, _xlpm.E_CH4 * _xlpm.GWP_CH4)</definedName>
     <definedName name="Common_Equations.Common_ConvertCH4ToCO2e_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 2, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"ECH4","Methane emissions (t CH4)";"GWPCH4","Global warming potential for methane (t CO2-e / t CH4)"}, _xlpm.r, _xlpm.c))))</definedName>
@@ -6318,9 +6315,10 @@
       <xdr:row>16</xdr:row>
       <xdr:rowOff>89047</xdr:rowOff>
     </xdr:to>
-    <xdr:sp macro="" textlink="'[1]4.3.1.1-2 Methane'!D27">
+    <xdr:sp macro="" textlink="'3.3.1.1-2 Enteric Methane'!D27">
       <xdr:nvSpPr>
         <xdr:cNvPr id="14" name="TextBox 13">
+          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D5DBF754-E65E-458F-A933-75ADD3406279}"/>
@@ -6365,7 +6363,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr algn="ctr"/>
-          <a:fld id="{63836C7B-CDBC-4017-8FDA-D8799018F3FC}" type="TxLink">
+          <a:fld id="{212D05B6-766E-4879-832C-4C68C5D13F73}" type="TxLink">
             <a:rPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike">
               <a:solidFill>
                 <a:srgbClr val="0D9D96"/>
@@ -6373,7 +6371,6 @@
               <a:latin typeface="Times New Roman"/>
               <a:cs typeface="Times New Roman"/>
             </a:rPr>
-            <a:pPr algn="ctr"/>
             <a:t>Milk production converted from milk solids</a:t>
           </a:fld>
           <a:endParaRPr lang="en-AU" sz="1000">
@@ -9141,56 +9138,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Home"/>
-      <sheetName val="Overview"/>
-      <sheetName val="Results"/>
-      <sheetName val="Input - Site"/>
-      <sheetName val="Input - Dairy"/>
-      <sheetName val="4.3.1.1-2 Methane"/>
-      <sheetName val="4.3.1.3-4 Direct N20"/>
-      <sheetName val="4.3.1.5 Atmos deposition"/>
-      <sheetName val="4.3.1.6-7 Leaching and runoff"/>
-      <sheetName val="4.3.1.8 Manure applied to soils"/>
-      <sheetName val="4.3.1.9 Soil direct N2O"/>
-      <sheetName val="4.3.1.10-11 Soil Atmos Dep"/>
-      <sheetName val="4.3.1.12-13 Soil leach runoff"/>
-      <sheetName val="Constants - Dairy"/>
-      <sheetName val="Constants - Common"/>
-      <sheetName val="Constants - Livestock"/>
-      <sheetName val="Acknowledgements"/>
-      <sheetName val="Tab template"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-      <sheetData sheetId="12"/>
-      <sheetData sheetId="13"/>
-      <sheetData sheetId="14"/>
-      <sheetData sheetId="15"/>
-      <sheetData sheetId="16"/>
-      <sheetData sheetId="17"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
 <rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
   <global>
@@ -25827,14 +25774,7 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAJwBSAGUAZgBlAHIAZQBuAGMAZQAnACwAIABhAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAGkAcwAgAGMAbwBuAHMAaQBzAHQAZQBuAHQAbAB5ACAAJwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdACcAIABhAG4AZAAgAGkAcwAgAG4AbwB0ACAAdQBzAGUAZAAgAGkAbgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAYgByAGUAZQBkAHMAXAAiACwAIAA2ADAAMAAsACAAMgAyADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAFcARwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAA1ADkAMAAsACAANQA5ADAALAAgADUAOQAwACwAIAA3ADcAMAAsACAANwA3ADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAHQAYQAgAGYAbwByACAAcAByAGUAIAAtACAAdwBlAGEAbgBlAGQAIABjAGEAbAB2AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAGoAPQAzACwANQA7ACAATgBQAFcAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagAnACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzADwAMQBcACIALAAgADAALgAwADEANwA2ACwAIAAwAC4AMgA2ADgANQAsACAAMAAuADAAMQAzADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzADwAMQBcACIALAAgADAALgAwADIAMAA0ACwAIAAwAC4AMwAwADAAMwAsACAAMAAuADAAMAA5ADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMQAwACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBOAFMAVwBcACIALAAgAFwAIgBOAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIAUwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAFYASQBDAFwAIgAsACAAXAAiAFcAQQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwAC4ANwAyACwAIAAwAC4ANwA2ACwAIAAwAC4AOAAsACAAMAAuADcAOAAsACAAMAAuADcANAAsACAAMAAuADYAOQAsACAAMAAuADcAMwAsACAAMAAuADcANgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AcwBcACIALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBzACAAKABhACkAXAAiACwAIAAwAC4AMQA1ACwAIAAwAC4AMQA4ACwAIAAwAC4ANQAwACwAIAAwAC4AMgA0ACwAIAAwAC4AMQA3ACwAIAAwAC4AMQAzACwAIAAwAC4AMQA3ACwAIAAwAC4AMQA4ACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQA7ACAARgByAGEAYwBHAEEAUwBNAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMQA3ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMgAwADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUgBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABNAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFIAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBSAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzACwAIABhAG4AZAAgAGgAbwB1AHMAZQAgAGMAbwB3AHMAXAAiACwAIAAxAC4AMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAG8AdABoAGUAcgAgAGMAYQB0AHQAbABlACAAYwBsAGEAcwBzAGUAcwBcACIALAAgADEALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABFAHgAYwBsAHUAZABlAGQAIAAnAEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQAnACAAcgBvAHcAIABhAHMAIAB0AGgAaQBzACAAaQBuAGYAbwByAG0AYQB0AGkAbwBuACAAaQBzACAAaQBuACAAdABoAGUAIAB0AGEAYgBsAGUAIAB0AGkAdABsAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHIAZQBhAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAFMAaABlAGQAXAAiACwAIABcACIARgBlAGUAZABwAGEAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAxADoAIABHAHIAYQB6AGUAZAAgAE8AbgBsAHkAXAAiACwAIAAwAC4AOAA5ACwAIAAwAC4AMQAxACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMgA6ACAATwBuACAAZgBlAGUAZABwAGEAZAAgAGYAbwByACAAPAAxADAAIABoAHIALwBkAGEAeQAgAGYAbwByACAAPAAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxACAAQQBuAGUAcgBvAGIAaQBjACAATABhAGcAbwBvAG4AXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAXAAiACwAIAAwACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADMAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAXAAiACwAIAAwACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0ANAAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABhAHkAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBvAG4AdgBlAHIAdABlAGQAIABmAHIAZQBlACAAdABlAHgAdAAgAGkAbgAgAGQAbwBjAHUAbQBlAG4AdAAgAHQAbwAgAHQAYQBiAGwAZQAsACAAbQBhAHQAYwBoAGkAbgBnACAAbABpAHYAZQBzAHQAbwBjAGsAIABjAGwAYQBzAHMAIABuAGEAbQBlAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKABwAHIAZQAtAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAXwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBEAFAAVwAnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABhACAAcwBlAHAAYQByAGEAdABlACAAaABhAG4AZABsAGkAbgBnACAAbwBmACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGQAdQByAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALABcAG4AIAAgACAAIAAyADAALgA3ACAAKgAgAEkAXwBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGEAcgBtAGwAZQB5ACAAZQB0ACAAYQBsAC4AIAAoADIAMAAxADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcAG4AVwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAXABuAEwAVwBHAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE0AUgBfAGoAIAA9ACAAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAE0ASQBfAGoAIAA9ACAAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVwBfAGoALAAgAEwAVwBHAF8AagAsACAATQBSAF8AagAsACAATQBJAF8AagAsAFwAbgAgACAAIAAgACgAMQAuADEAOAA1ACAAKwAgADAALgAwADAANAA1ADQAIAAqACAAVwBfAGoAIAAtACAAMAAuADAAMAAwADAAMAAyADYAIAAqACAAVwBfAGoAIABeACAAMgAgACsAIAAwAC4AMwAxADUAIAAqACAATABXAEcAXwBqACkAIABeACAAMgAgACoAIABNAFIAXwBqACAAKwAgAE0ASQBfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBrAGcAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAFcARwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBSAF8AagBcACIALAAgAFwAIgBpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ASQBfAGoAXAAiACwAIABcACIAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBNAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAE0ASQBfAGoAPQAoAE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQApAC8AKABHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagApAFwAbgBNAFAAXwBqACAAPQAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABMAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE4ARQAgAD0AIABuAGUAdAAgAGUAbgBlAHIAZwB5ACAAKABNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawApAFwAbgBHAEUAQwAgAD0AIABnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIAAoAE0ASgAvAGsAZwBEAE0AKQBcAG4AawAgAD0AIABlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4AcQBtAF8AagAgAD0AIABtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBQAF8AagAsACAATgBFACwAIABHAEUAQwAsACAAawAsACAAcQBtAF8AagAsAFwAbgAgACAAIAAgACgATQBQAF8AagAgACoAIAAxAC4AMAAzACAAKgAgAE4ARQApACAALwAgACgARwBFAEMAIAAqACAAawAgACoAIABxAG0AXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagA9AFwAXABmAHIAYQBjAHsATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFAH0AewBHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBcACIALAAgAFwAIgBuAGUAdAAgAGUAbgBlAHIAZwB5AFwAIgAsACAAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBFAEMAXAAiACwAIABcACIAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0AFwAIgAsACAAXAAiAE0ASgAvAGsAZwBEAE0AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBrAFwAIgAsACAAXAAiAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBtAF8AagBcACIALAAgAFwAIgBtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADYAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4ATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXABuAE0AUABfAGoAXABuAEwALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AUABfAGoAPQBNAFMAXwBqAC8AKAAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAKQBcAG4ATQBTAF8AagAgAD0AIABkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAKABrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgBDAF8AagAgAD0AIABmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAFAAQwBfAGoAIAA9ACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBTAF8AagAsACAARgBDAF8AagAsACAAUABDAF8AagAsAFwAbgAgACAAIAAgAE0AUwBfAGoAIAAvACAAKAAwAC4AMAAxACAAKgAgACgARgBDAF8AagAgACsAIABQAEMAXwBqACkAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAPQBcAFwAZgByAGEAYwB7AE0AUwBfAGoAfQB7ADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgAgAEMAbwBuAHYAZQByAHQAZQBkACAAaQBuAHAAdQB0ACAARgBDACAAYQBuAGQAIABQAEMAIABwAGUAcgBjAGUAbgB0ACAAdABvACAAaQBuAHQAZQBnAGUAcgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAbgBxAG0AXwBqAFwAbgBmAHIAYQBjAHQAaQBvAG4AXABuAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4ANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAATQBNAFMARgByAGEAYwB0AGkAbwBuACwAIABGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgATQBNAFMARgByAGEAYwB0AGkAbwBuAC0AKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4AKgBGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQAKQApAFwAbgApADsAXABuAFwAbgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACwAXABuACAAIAAgACAATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25847,7 +25787,14 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGsAZwApACAALQAgAEMAbwB3AHMAIABhAG4AZAAgAEgAZQBpAGYAZQByAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQwBvAHcAcwAgAGEAbgBkACAASABlAGkAZgBlAHIAcwAgACgAVwBqACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAARQB4AGMAbAB1AGQAZQBkACAAJwBSAGUAZgBlAHIAZQBuAGMAZQAnACwAIABhAHMAIAB0AGgAZQAgAHYAYQBsAHUAZQAgAGkAcwAgAGMAbwBuAHMAaQBzAHQAZQBuAHQAbAB5ACAAJwBEAGEAaQByAHkAIABBAHUAcwB0AHIAYQBsAGkAYQAgAFsAMQBdACcAIABhAG4AZAAgAGkAcwAgAG4AbwB0ACAAdQBzAGUAZAAgAGkAbgAgAGMAYQBsAGMAdQBsAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAxACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAcgBlAGUAZABcACIALAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AZQBkAGkAdQBtACAARgByAGkAZQBzAGkAYQBuAFwAIgAsACAANQA1ADAALAAgADMAOAAwACwAIAAxADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGEAcgBnAGUAIABGAHIAaQBlAHMAaQBhAG4AXAAiACwAIAA2ADAAMAAsACAANAAxADUALAAgADEANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwBsAHMAdABlAGkAbgAtAEYAcgBpAGUAcwBpAGEAbgBcACIALAAgADYANQAwACwAIAA0ADUAMAAsACAAMQA4ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGkAZQBzAGkAYQBuACAAYwByAG8AcwBzAGIAcgBlAGQAXAAiACwAIAA1ADAAMAAsACAAMwA1ADAALAAgADEANAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAZQByAHMAZQB5AFwAIgAsACAANAAwADAALAAgADIANwA1ACwAIAAxADEANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGUAcgBzAGUAeQAgAGMAcgBvAHMAcwBiAHIAZQBkAFwAIgAsACAANAA1ADAALAAgADMAMQA1ACwAIAAxADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHkAcgBzAGgAaQByAGUAXAAiACwAIAA1ADQAMAAsACAAMwA3ADUALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAdQBlAHIAbgBzAGUAeQBcACIALAAgADQAOAAwACwAIAAzADMANQAsACAAMQA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAG8AdwBuACAAUwB3AGkAcwBzAFwAIgAsACAANgAwADAALAAgADQAMQA1ACwAIAAxADcAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAGwAbABhAHcAYQByAHIAYQAvAEEAdQBzAHMAaQBlACAAUgBlAGQAXAAiACwAIAA1ADUAMAAsACAAMwA3ADUALAAgADEANQAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgAyADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQAgAC0AIABCAHUAbABsAHMAIAAoAFcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AMgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAIAAtACAAQgB1AGwAbABzACAAKABXAGoAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBXAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgByAGUAZQBkAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgAD4AMQBcACIALAAgAFwAIgBCAHUAbABsAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABsACAAYgByAGUAZQBkAHMAXAAiACwAIAA2ADAAMAAsACAAMgAyADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAIABnAGEAaQBuACAAKABrAGcAKQAgACgATABXAEcAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAFcARwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAwAC4AMAAxADYALAAgADAALgA2ACwAIAAwAC4ANQA3ACwAIAAwAC4AMQAsACAAMAAuADgAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0ADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABSAGUAZgBlAHIAZQBuAGMAZQAgAHcAZQBpAGcAaAB0AHMAIAAoAGsAZwApACAAKABXAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBSAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADMALgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAbABrAGkAbgBnACAAQwBvAHcAcwBcACIALAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPgAxAFwAIgAsACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ADEAIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIAQgB1AGwAbABzACAAPgAxAFwAIgAsACAAXAAiAEIAdQBsAGwAcwAgADwAMQAgACgAdwBlAGEAbgBlAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAA1ADkAMAAsACAANQA5ADAALAAgADUAOQAwACwAIAA3ADcAMAAsACAANwA3ADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAHQAYQAgAGYAbwByACAAcAByAGUAIAAtACAAdwBlAGEAbgBlAGQAIABjAGEAbAB2AGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEQAYQB0AGEAIABmAG8AcgAgAHAAcgBlACAALQAgAHcAZQBhAG4AZQBkACAAYwBhAGwAdgBlAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBTAGoAPQAzACwANQA7ACAATgBQAFcAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIAAnAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagAnACAAYwBvAGwAdQBtAG4AIABoAGUAYQBkAGUAcgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGkAbQBhAGwAIABjAGwAYQBzAHMAIABqAFwAIgAsACAAXAAiAEMASAA0ACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgACgAVgBTAGoAPQAzACwANQApAFwAIgAsACAAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAEUAeABjAHIAZQB0AGUAZAAgACgATgBQAFcAagA9ADMALAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiACgAawBnAC8AZABhAHkAKQBcACIALAAgAFwAIgAoAGsAZwAvAGQAYQB5ACkAXAAiACwAIABcACIAKABrAGcALwBkAGEAeQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzADwAMQBcACIALAAgADAALgAwADEANwA2ACwAIAAwAC4AMgA2ADgANQAsACAAMAAuADAAMQAzADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzADwAMQBcACIALAAgADAALgAwADIAMAA0ACwAIAAwAC4AMwAwADAAMwAsACAAMAAuADAAMAA5ADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGoAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4ANgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMQAwACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBBAEMAVABcACIALAAgAFwAIgBOAFMAVwBcACIALAAgAFwAIgBOAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIAUwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAFYASQBDAFwAIgAsACAAXAAiAFcAQQBcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIAAwAC4ANwAyACwAIAAwAC4ANwA2ACwAIAAwAC4AOAAsACAAMAAuADcAOAAsACAAMAAuADcANAAsACAAMAAuADYAOQAsACAAMAAuADcAMwAsACAAMAAuADcANgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AcwBcACIALAAgADAALgAwADAANQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADAANQAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAALQAgAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawBzACAAKABhACkAXAAiACwAIAAwAC4AMQA1ACwAIAAwAC4AMQA4ACwAIAAwAC4ANQAwACwAIAAwAC4AMgA0ACwAIAAwAC4AMQA3ACwAIAAwAC4AMQAzACwAIAAwAC4AMQA3ACwAIAAwAC4AMQA4ACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAMAAuADAAMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGEAbgBkACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQA7ACAARgByAGEAYwBHAEEAUwBNAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZQB4AGMAcgBlAHQAZQBkAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARQBGAG0AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABlAHgAYwByAGUAdABlAGQAKQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGUAeABjAHIAZQB0AGUAZAApAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAxACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAD0AMgAgAEQAYQBpAGwAeQAgAFMAcAByAGUAYQBkACAALQAgAFMAdQBtAHAAIABhAG4AZAAgAEQAaQBzAHAAZQByAHMAYQBsAFwAIgAsACAAMAAsACAAMAAuADAANwAsACAAXAAiAFMAdQBtAHAAIABhAG4AZAAgAGQAaQBzAHAAZQByAHMAYQBsACAAcwB5AHMAdABlAG0AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAARABhAGkAbAB5ACAAUwBwAHIAZQBhAGQAIAAtACAARAByAGEAaQBuAHMAIAB0AG8AIABQAGEAZABkAG8AYwBrAFwAIgAsACAAMAAsACAAMAAuADIALAAgAFwAIgBEAHIAYQBpAG4AcwAgAHQAbwAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0APQAzACAAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQBcACIALAAgADAALgAwADAANQAsACAAMAAuADMALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADgAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAE0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQAgACgATQBQAFcARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AOABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAQwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBNAFAAVwBFAE4AVABFAFIASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGUAaQBmAGUAcgBzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMQA3ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGwAbABzACAAPAAgADEAIAB5AGUAYQByAFwAIgAsACAAMAAuADAAMgAwADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAOgAgAEQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAALQAgAEkAbgBjAHIAZQBhAHMAZQBkACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAE0AUgBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABhAGIAbABlACAAQQAuADEALgAzAC4AOQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAASQBuAGMAcgBlAGEAcwBlAGQAIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrACAAKABNAFIAagApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAFIAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AaQBtAGEAbAAgAEMAbABhAHMAcwAgAGoAXAAiACwAIABcACIATQBSAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzACwAIABhAG4AZAAgAGgAbwB1AHMAZQAgAGMAbwB3AHMAXAAiACwAIAAxAC4AMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAbAAgAG8AdABoAGUAcgAgAGMAYQB0AHQAbABlACAAYwBsAGEAcwBzAGUAcwBcACIALAAgADEALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBcAG4AVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwADoAIABEAGEAaQByAHkAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHYAbwBpAGQAZQBkACAAdABvACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBNAFMAagBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMAA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB2AG8AaQBkAGUAZAAgAHQAbwAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAGoAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAagBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABFAHgAYwBsAHUAZABlAGQAIAAnAEEAbgBuAHUAYQBsACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdABpAG0AZQAgAHMAcABlAG4AdAAgAHAAZQByACAAYQByAGUAYQAnACAAcgBvAHcAIABhAHMAIAB0AGgAaQBzACAAaQBuAGYAbwByAG0AYQB0AGkAbwBuACAAaQBzACAAaQBuACAAdABoAGUAIAB0AGEAYgBsAGUAIAB0AGkAdABsAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHIAZQBhAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATQBpAGwAawBpAG4AZwAgAFMAaABlAGQAXAAiACwAIABcACIARgBlAGUAZABwAGEAZABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAAxADoAIABHAHIAYQB6AGUAZAAgAE8AbgBsAHkAXAAiACwAIAAwAC4AOAA5ACwAIAAwAC4AMQAxACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAeQBzAHQAZQBtACAAMgA6ACAATwBuACAAZgBlAGUAZABwAGEAZAAgAGYAbwByACAAPAAxADAAIABoAHIALwBkAGEAeQAgAGYAbwByACAAPAAzACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADcAOQAsACAAMAAuADEAMQAsACAAMAAuADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHkAcwB0AGUAbQAgADMAOgAgAFAAYQBzAHQAdQByAGUALQBnAHIAYQB6AGUAZAAgADMALQA5ACAAbQBvAG4AdABoAHMALwB5AGUAYQByAFwAIgAsACAAMAAuADUAMwA0ACwAIAAwAC4AMQAxACwAIAAwAC4AMwA1ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AHMAdABlAG0AIAA0ADoAIABaAGUAcgBvACAAZwByAGEAegBpAG4AZwBcACIALAAgADAALAAgADAALgAxADEALAAgADAALgA4ADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgAEEALgAxAC4AMwAuADEAMQA6ACAARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIAAtACAARQBGACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAcABlAHIAIABNAE0AUwAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAbQApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAzAC4AMQAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAOgAgAEEAZABkAGUAZAAgACcATgBJAFIAIAByAGUAZgBlAHIAZQBuAGMAZQAnACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxADQAIABQAGEAcwB0AHUAcgBlAFwAIgAsACAAMAAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAG0APQAxACAAQQBuAGUAcgBvAGIAaQBjACAATABhAGcAbwBvAG4AXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADIAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAXAAiACwAIAAwACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAbQA9ADMAIABEAGEAaQBsAHkAIABTAHAAcgBlAGEAZAA6ACAARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAHMAXAAiACwAIAAwACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAD0ANAAgAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAZgBvAHIAIABlAGEAYwBoACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AcAB1AHQAIABjAGwAYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAGYAbwByACAAZQBhAGMAaAAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuAHAAdQB0ACAAYwBsAGEAcwBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABhAHkAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQA6ACAAQwBvAG4AdgBlAHIAdABlAGQAIABmAHIAZQBlACAAdABlAHgAdAAgAGkAbgAgAGQAbwBjAHUAbQBlAG4AdAAgAHQAbwAgAHQAYQBiAGwAZQAsACAAbQBhAHQAYwBoAGkAbgBnACAAbABpAHYAZQBzAHQAbwBjAGsAIABjAGwAYQBzAHMAIABuAGEAbQBlAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBpAG0AYQBsACAAYwBsAGEAcwBzACAAagBcACIALAAgAFwAIgBEAHUAcgBhAHQAaQBvAG4AIAAoAHcAZQBhAG4AZQBkACkAXAAiACwAIABcACIARAB1AHIAYQB0AGkAbwBuACAAKABwAHIAZQAtAHcAZQBhAG4AZQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBsAGsAaQBuAGcAIABjAG8AdwBzAFwAIgAsACAAMwA2ADUALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABlAGkAZgBlAHIAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAZQBpAGYAZQByAHMAIAA8ACAAMQAgAHkAZQBhAHIAXAAiACwAIAAyADgAMQAsACAAOAA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgAD4AIAAxACAAeQBlAGEAcgBcACIALAAgADMANgA1ACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBsAGwAcwAgADwAIAAxACAAeQBlAGEAcgBcACIALAAgADIAOAAxACwAIAA4ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXABuAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBQAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcAG4ARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABNAEQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyAFwAdABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADcANQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AFwAbgBOAGUAdAAgAGUAbgBlAHIAZwB5ACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AZQB0ACAAZQBuAGUAcgBnAHkAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ARQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBKACAAbgBlAHQAIABlAG4AZQByAGcAeQAgAC8AIABrAGcAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMwAuADAANQA0ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXABuAEcAcgBvAHMAcwAgAGUAbgBlAHIAZwB5ACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAGYAZQBlAGQAIABkAHIAeQAgAG0AYQB0AHQAZQByAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgAGQAcgB5ACAAbQBhAHQAdABlAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBFAEMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ASgAgAC8AIABrAGcARABNAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMQA4AC4ANAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AFwAbgBFAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAdQBzAGUAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBmAGYAaQBjAGkAZQBuAGMAeQAgAG8AZgAgAHUAcwBlACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAA4ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4AQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBfAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQALwBrAGcAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADIANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBGAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAzAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAxADEAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAXwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADMALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHoAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQB6AGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBcAG4ARgBhAHQAIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQB0ACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBDAF8AagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADIALgAyACAARABBAFQAQQAgACgATQBFAFQASABPAEQAIAAxACAAQQBOAEQAIAAyACAATwBQAFQASQBPAE4AUwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADQALgAwACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAFwAbgBQAHIAbwB0AGUAaQBuACAAYwBvAG4AdABlAG4AdAAgAGkAbgAgAGYAYQB0ACAAYQBuAGQAIABwAHIAbwB0AGUAaQBuACAAYwBvAHIAcgBlAGMAdABlAGQAIABtAGkAbABrAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAQwBfAGoAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBwAGUAcgBjAGUAbgB0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMgAuADIAIABEAEEAVABBACAAKABNAEUAVABIAE8ARAAgADEAIABBAE4ARAAgADIAIABPAFAAVABJAE8ATgBTACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADMALgAzACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMwA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARABhAGkAcgB5ACAAQwBhAHQAdABsAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAzAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEQAYQBpAHIAeQAgAEMAYQB0AHQAbABlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABkAGEAaQByAHkAIABjAGEAdAB0AGwAZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AKAAoAE4AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMQAsADIALAA0AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAD0AMwAsADUAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBQAFcAXwB7AEUATgBUAEUAUgBJAEMALABqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAxADIANAAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGgAZQBhAGQAKQBcAG4ATQBfAGoAMQAyADQAIAA9ACAAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANAAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARABfAGoAMQAyADQAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAIAAoAGQAYQB5AHMAKQBcAG4ATgBfAGoAMwA1ACAAPQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABoAGUAYQBkACkAXABuAE0AXwBqADMANQAgAD0AIABkAGEAaQBsAHkAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAG8AcgAgAGMAbABhAHMAcwBlAHMAIABqAD0AMwAsADUAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqADMANQAgAD0AIABkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBuACAAdABoAGUAIABmAGEAcgBtACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1ACAAKABkAGEAeQBzACkAXABuAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABwAHIAZQAtAHcAZQBhAG4AZQBkACAAaABlAGkAZgBlAHIAIABhAG4AZAAgAGIAdQBsAGwAIABjAGEAbAB2AGUAcwAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqADEAMgA0ACwAIABNAF8AagAxADIANAAsACAARABfAGoAMQAyADQALAAgAE4AXwBqADMANQAsACAATQBfAGoAMwA1ACwAIABEAF8AagAzADUALAAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACwAXABuACAAIAAgACAAKAAoAE4AXwBqADEAMgA0ACAAKgAgAE0AXwBqADEAMgA0ACAAKgAgAEQAXwBqADEAMgA0ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACAAKwAgACgATgBfAGoAMwA1ACAAKgAgAE0AUABXAF8ARQBOAFQARQBSAEkAQwBfAGoAMwA1ACAAKgAgAEQAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoAMQAyADQALAAgAE0AXwBqADEAMgA0ACwAIABEAF8AagAxADIANAAsACAATgBfAGoAMwA1ACwAIABNAF8AagAzADUALAAgAEQAXwBqADMANQAsACAARABQAFcAXwBqADMANQAsACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUALABcAG4AIAAgACAAIAAoACgATgBfAGoAMQAyADQAIAAqACAATQBfAGoAMQAyADQAIAAqACAARABfAGoAMQAyADQAKQAgACsAIAAoAE4AXwBqADMANQAgACoAIABNAF8AagAzADUAIAAqACAARABfAGoAMwA1ACkAIAArACAAKABOAF8AagAzADUAIAAqACAATQBQAFcAXwBFAE4AVABFAFIASQBDAF8AagAzADUAIAAqACAARABQAFcAXwBqADMANQApACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAzAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgAKABOAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAPQAxACwAMgAsADQAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADEALAAyACwANAB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagA9ADMALAA1AH0AKQArACgATgBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAE0AUABXAF8AewBFAE4AVABFAFIASQBDACwAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoACgATgBfAHsAagA9ADEALAAyACwANAB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAD0AMQAsADIALAA0AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAxACwAMgAsADQAfQApACsAKABOAF8AewBqAD0AMwAsADUAfQBcAFwAdABpAG0AZQBzACAATQBfAHsAagA9ADMALAA1AH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAPQAzACwANQB9ACkAKwAoAE4AXwB7AGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABNAFAAVwBfAHsARQBOAFQARQBSAEkAQwAsAGoAPQAzACwANQB9AFwAXAB0AGkAbQBlAHMAIABEAFAAVwBfAHsAagA9ADMALAA1AH0AKQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADEAMgA0AFwAIgAsACAAXAAiAG4AdQBtAGIAZQByACAAbwBmACAAZABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABpAG4AIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMQAyADQAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgBvAHIAIABjAGwAYQBzAHMAZQBzACAAagA9ADEALAAyACwANABcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAMQAyADQAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAxACwAMgAsADQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqADMANQBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQBpAHIAeQAgAGMAYQB0AHQAbABlACAAaQBuACAAYwBsAGEAcwBzAGUAcwAgAGoAPQAzACwANQBcACIALAAgAFwAIgBoAGUAYQBkAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAMwA1AFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADMALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAF8AagAzADUAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AbgAgAHQAaABlACAAZgBhAHIAbQAgAGYAbwByACAAdwBlAGEAbgBlAGQAIABjAGwAYQBzAHMAZQBzACAAagA9ADMALAA1AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAFAAVwBfAGoAMwA1AFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAG4AIAB0AGgAZQAgAGYAYQByAG0AIABmAG8AcgAgAHAAcgBlAC0AdwBlAGEAbgBlAGQAIABoAGUAaQBmAGUAcgAgAGEAbgBkACAAYgB1AGwAbAAgAGMAYQBsAHYAZQBzAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVwBfAEUATgBUAEUAUgBJAEMAXwBqADMANQBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAbwByACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGgAZQBpAGYAZQByACAAYQBuAGQAIABiAHUAbABsACAAYwBhAGwAdgBlAHMAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAJwBEAFAAVwAnACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABhACAAcwBlAHAAYQByAGEAdABlACAAaABhAG4AZABsAGkAbgBnACAAbwBmACAAcAByAGUALQB3AGUAYQBuAGUAZAAgAGQAdQByAGEAdABpAG8AbgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABmAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAoAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALABcAG4AIAAgACAAIAAyADAALgA3ACAAKgAgAEkAXwBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGEAcgBtAGwAZQB5ACAAZQB0ACAAYQBsAC4AIAAoADIAMAAxADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AMgAwAC4ANwBcAFwAdABpAG0AZQBzACAASQBfAGoAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAAzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcAG4ASQBfAGoAXABuAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcAG4ASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcAG4AVwBfAGoAIAA9ACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAawBnACkAXABuAEwAVwBHAF8AagAgAD0AIABsAGkAdgBlAHcAZQBpAGcAaAB0ACAAZwBhAGkAbgAgACgAawBnAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE0AUgBfAGoAIAA9ACAAaQBuAGMAcgBlAGEAcwBlACAAaQBuACAAbQBlAHQAYQBiAG8AbABpAGMAIAByAGEAdABlACAAdwBoAGUAbgAgAHAAcgBvAGQAdQBjAGkAbgBnACAAbQBpAGwAawAgACgAZgByAGEAYwB0AGkAbwBuACkAXABuAE0ASQBfAGoAIAA9ACAAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVwBfAGoALAAgAEwAVwBHAF8AagAsACAATQBSAF8AagAsACAATQBJAF8AagAsAFwAbgAgACAAIAAgACgAMQAuADEAOAA1ACAAKwAgADAALgAwADAANAA1ADQAIAAqACAAVwBfAGoAIAAtACAAMAAuADAAMAAwADAAMAAyADYAIAAqACAAVwBfAGoAIABeACAAMgAgACsAIAAwAC4AMwAxADUAIAAqACAATABXAEcAXwBqACkAIABeACAAMgAgACoAIABNAFIAXwBqACAAKwAgAE0ASQBfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBfAGoAPQAoADEALgAxADgANQArADAALgAwADAANAA1ADQAXABcAHQAaQBtAGUAcwAgAFcAXwBqAC0AMAAuADAAMAAwADAAMAAyADYAXABcAHQAaQBtAGUAcwAgAFcAXwBqAF4AMgArADAALgAzADEANQBcAFwAdABpAG0AZQBzACAATABXAEcAXwBqACkAXgAyAFwAXAB0AGkAbQBlAHMAIABNAFIAXwBqACsATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBrAGcAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAFcARwBfAGoAXAAiACwAIABcACIAbABpAHYAZQB3AGUAaQBnAGgAdAAgAGcAYQBpAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBSAF8AagBcACIALAAgAFwAIgBpAG4AYwByAGUAYQBzAGUAIABpAG4AIABtAGUAdABhAGIAbwBsAGkAYwAgAHIAYQB0AGUAIAB3AGgAZQBuACAAcAByAG8AZAB1AGMAaQBuAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ASQBfAGoAXAAiACwAIABcACIAYQBkAGQAaQB0AGkAbwBuAGEAbAAgAGkAbgB0AGEAawBlACAAcgBlAHEAdQBpAHIAZQBkACAAZgBvAHIAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA0ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBBAGQAZABpAHQAaQBvAG4AYQBsACAAaQBuAHQAYQBrAGUAIAByAGUAcQB1AGkAcgBlAGQAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBNAEkAXwBqAFwAbgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXABuAE0ASQBfAGoAPQAoAE0AUABfAGoAXABcAHQAaQBtAGUAcwAgADEALgAwADMAXABcAHQAaQBtAGUAcwAgAE4ARQApAC8AKABHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagApAFwAbgBNAFAAXwBqACAAPQAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABMAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAE4ARQAgAD0AIABuAGUAdAAgAGUAbgBlAHIAZwB5ACAAKABNAEoAIABuAGUAdAAgAGUAbgBlAHIAZwB5AC8AawBnACAAbQBpAGwAawApAFwAbgBHAEUAQwAgAD0AIABnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgAGMAbwBuAHQAZQBuAHQAIAAoAE0ASgAvAGsAZwBEAE0AKQBcAG4AawAgAD0AIABlAGYAZgBpAGMAaQBlAG4AYwB5ACAAbwBmACAAbQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQAgAGUAbgBlAHIAZwB5ACAAdQBzAGUAIABmAG8AcgAgAG0AaQBsAGsAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4AcQBtAF8AagAgAD0AIABtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0ACAAKABmAHIAYQBjAHQAaQBvAG4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBQAF8AagAsACAATgBFACwAIABHAEUAQwAsACAAawAsACAAcQBtAF8AagAsAFwAbgAgACAAIAAgACgATQBQAF8AagAgACoAIAAxAC4AMAAzACAAKgAgAE4ARQApACAALwAgACgARwBFAEMAIAAqACAAawAgACoAIABxAG0AXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAZABkAGkAdABpAG8AbgBhAGwAIABpAG4AdABhAGsAZQAgAHIAZQBxAHUAaQByAGUAZAAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBJAF8AagA9AFwAXABmAHIAYQBjAHsATQBQAF8AagBcAFwAdABpAG0AZQBzACAAMQAuADAAMwBcAFwAdABpAG0AZQBzACAATgBFAH0AewBHAEUAQwBcAFwAdABpAG0AZQBzACAAawBcAFwAdABpAG0AZQBzACAAcQBtAF8AagB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAFUAXAAiACwAIABcACIAaQBuAHAAdQB0ACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0AFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBQAF8AagBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAaQBmACAAaQBuAHAAdQB0ACAAYQBzACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrACkAXAAiACwAIABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AUABfAGoAXAAiACwAIABcACIAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAAoAGkAZgAgAGkAbgBwAHUAdAAgAGEAcwAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwApAFwAIgAsACAAXAAiAEwALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMwAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBcACIALAAgAFwAIgBuAGUAdAAgAGUAbgBlAHIAZwB5AFwAIgAsACAAXAAiAE0ASgAgAG4AZQB0ACAAZQBuAGUAcgBnAHkALwBrAGcAIABtAGkAbABrAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBFAEMAXAAiACwAIABcACIAZwByAG8AcwBzACAAZQBuAGUAcgBnAHkAIABjAG8AbgB0AGUAbgB0AFwAIgAsACAAXAAiAE0ASgAvAGsAZwBEAE0AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBrAFwAIgAsACAAXAAiAGUAZgBmAGkAYwBpAGUAbgBjAHkAIABvAGYAIABtAGUAdABhAGIAbwBsAGkAegBhAGIAbABlACAAZQBuAGUAcgBnAHkAIAB1AHMAZQAgAGYAbwByACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcQBtAF8AagBcACIALAAgAFwAIgBtAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAdABoAGUAIABkAGkAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAzAC4AMQAuADEAIAAoADYAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAbQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIAB1AG4AaQB0ACAAdgBhAHIAaQBhAGIAbABlACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIAB1AHMAZQAgAG8AZgAgAGUAaQB0AGgAZQByACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAbwByACAAbABpAHQAcgBlAHMAIABvAGYAIABtAGkAbABrAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBcAG4ATQBpAGwAawAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABjAG8AbgB2AGUAcgB0AGUAZAAgAGYAcgBvAG0AIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXABuAE0AUABfAGoAXABuAEwALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AUABfAGoAPQBNAFMAXwBqAC8AKAAwAC4AMAAxAFwAXAB0AGkAbQBlAHMAIAAoAEYAQwBfAGoAKwBQAEMAXwBqACkAKQBcAG4ATQBTAF8AagAgAD0AIABkAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBpAGwAawAgAHMAbwBsAGkAZABzACAAKABrAGcAIABNAFMALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgBDAF8AagAgAD0AIABmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAFAAQwBfAGoAIAA9ACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBTAF8AagAsACAARgBDAF8AagAsACAAUABDAF8AagAsAFwAbgAgACAAIAAgAE0AUwBfAGoAIAAvACAAKAAwAC4AMAAxACAAKgAgACgARgBDAF8AagAgACsAIABQAEMAXwBqACkAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGMAbwBuAHYAZQByAHQAZQBkACAAZgByAG8AbQAgAG0AaQBsAGsAIABzAG8AbABpAGQAcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADMALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AUABfAGoAPQBcAFwAZgByAGEAYwB7AE0AUwBfAGoAfQB7ADAALgAwADEAXABcAHQAaQBtAGUAcwAgACgARgBDAF8AagArAFAAQwBfAGoAKQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBpAG4AcAB1AHQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFAAVQBcACIALAAgAFwAIgBtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAFMAXwBqAFwAIgAsACAAXAAiAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAXAAiACwAIABcACIAawBnACAATQBTAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBDAF8AagBcACIALAAgAFwAIgBmAGEAdAAgAGMAbwBuAHQAZQBuAHQAIABpAG4AIABmAGEAdAAgAGEAbgBkACAAcAByAG8AdABlAGkAbgAgAGMAbwByAHIAZQBjAHQAZQBkACAAbQBpAGwAawBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEMAXwBqAFwAIgAsACAAXAAiAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAaQBuACAAZgBhAHQAIABhAG4AZAAgAHAAcgBvAHQAZQBpAG4AIABjAG8AcgByAGUAYwB0AGUAZAAgAG0AaQBsAGsAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABBAGQAZABlAGQAIABtAGkAbABrACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAHUAbgBpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIAB0AG8AIABhAGwAbABvAHcAIABmAG8AcgAgAHUAcwBlACAAbwBmACAAZQBpAHQAaABlAHIAIABtAGkAbABrACAAcwBvAGwAaQBkAHMAIABvAHIAIABsAGkAdAByAGUAcwAgAG8AZgAgAG0AaQBsAGsALgAgAEMAbwBuAHYAZQByAHQAZQBkACAAaQBuAHAAdQB0ACAARgBDACAAYQBuAGQAIABQAEMAIABwAGUAcgBjAGUAbgB0ACAAdABvACAAaQBuAHQAZQBnAGUAcgAuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXABuAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkAIABvAGYAIABkAGkAZQB0AFwAbgBxAG0AXwBqAFwAbgBmAHIAYQBjAHQAaQBvAG4AXABuAHEAbQBfAGoAPQAwAC4ANwA5ADUAXABcAHQAaQBtAGUAcwAgACgARABNAEQAXwBqAFwAXAB0AGkAbQBlAHMAIAAxADAAMAApAC0AMAAuADAAMAAxADQAXABuAEQATQBEAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAE0ARABfAGoALABcAG4AIAAgACAAIAAwAC4ANwA5ADUAIAAqACAAKABEAE0ARABfAGoAIAAqACAAMQAwADAAKQAgAC0AIAAwAC4AMAAwADEANABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5ACAAbwBmACAAZABpAGUAdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHEAbQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcQBtAF8AagA9ADAALgA3ADkANQBcAFwAdABpAG0AZQBzACAAKABEAE0ARABfAGoAXABcAHQAaQBtAGUAcwAgADEAMAAwACkALQAwAC4AMAAwADEANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABNAEQAXwBqAFwAIgAsACAAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZQB4AHAAcgBlAHMAcwBlAGQAIABhAHMAIABhACAAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAiACwAIgB0AGUAeAB0ACIAOgAiAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAATQBNAFMARgByAGEAYwB0AGkAbwBuACwAIABGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACAAKgAgACgATQBNAFMARgByAGEAYwB0AGkAbwBuAC0AKABNAE0AUwBGAHIAYQBjAHQAaQBvAG4AKgBGAHIAYQBjAHQAaQBvAG4AUwBlAHAAYQByAGEAdABlAGQAKQApAFwAbgApADsAXABuAFwAbgBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQBuAGkAdABhAGwAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUARgByAGEAYwB0AGkAbwBuACwAXABuACAAIAAgACAATQBNAFMAMQBGAHIAYQBjAHQAaQBvAG4ALAAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQALAAgAFwAbgAgACAAIAAgAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACwAIABNAE0AUwAyAFMAZQBwAGEAcgBhAHQAZQBkACwAIABcAG4AIAAgACAAIABNAE0AUwAzAEYAcgBhAGMAdABpAG8AbgAsACAATQBNAFMAMwBTAGUAcABhAHIAYQB0AGUAZAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AIAAqACAAKABcAG4AIAAgACAAIAAgACAAIAAgAEkAbgBpAHQAYQBsAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAEYAcgBhAGMAdABpAG8AbgAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADEARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADEAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADIARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADIAUwBlAHAAYQByAGEAdABlAGQAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAoAE0ATQBTADMARgByAGEAYwB0AGkAbwBuACAAKgAgAE0ATQBTADMAUwBlAHAAYQByAGEAdABlAGQAKQBcAG4AIAAgACAAIAApAFwAbgApADsAIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUASABhAHIAdgBlAHMAdABJAG4AZABlAHgAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQwBvAHcAcwBBAG4AZABIAGUAaQBmAGUAcgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEMAbwB3AHMAQQBuAGQASABlAGkAZgBlAHIAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABDAG8AdwBzAEEAbgBkAEgAZQBpAGYAZQByAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQAQgB1AGwAbABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEIAdQBsAGwAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABCAHUAbABsAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEwAaQB2AGUAdwBlAGkAZwBoAHQARwBhAGkAbgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATABpAHYAZQB3AGUAaQBnAGgAdABHAGEAaQBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBMAGkAdgBlAHcAZQBpAGcAaAB0AEcAYQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUgBlAGYAZQByAGUAbgBjAGUAVwBlAGkAZwBoAHQAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBSAGUAZgBlAHIAZQBuAGMAZQBXAGUAaQBnAGgAdABzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFIAZQBmAGUAcgBlAG4AYwBlAFcAZQBpAGcAaAB0AHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBDAEYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAEEAbgBkAEYAcgBhAGMARwBBAFMATQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAQQBuAGQARgByAGEAYwBHAEEAUwBNAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBBAG4AZABGAHIAYQBjAEcAQQBTAE0AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAHIAZQBXAGUAYQBuAGUAZABDAGEAbAB2AGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAcgBlAFcAZQBhAG4AZQBkAEMAYQBsAHYAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUAByAGUAVwBlAGEAbgBlAGQAQwBhAGwAdgBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEkAbgBjAHIAZQBhAHMAZQBkAE0AZQB0AGEAYgBvAGwAaQBjAFIAYQB0AGUATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ASQBuAGMAcgBlAGEAcwBlAGQATQBlAHQAYQBiAG8AbABpAGMAUgBhAHQAZQBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBJAG4AYwByAGUAYQBzAGUAZABNAGUAdABhAGIAbwBsAGkAYwBSAGEAdABlAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBWAG8AaQBkAGUAZABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFYAbwBpAGQAZQBkAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVgBvAGkAZABlAGQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUARgBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBQAGUAcgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBGAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAFAAZQByAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAEYATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUAUABlAHIATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEMAcgB1AGQAZQBQAHIAbwB0AGUAaQBuAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBDAHIAdQBkAGUAUAByAG8AdABlAGkAbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQwByAHUAZABlAFAAcgBvAHQAZQBpAG4AXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARAByAHkATQBhAHQAdABlAHIARABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBEAHIAeQBNAGEAdAB0AGUAcgBEAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEQAcgB5AE0AYQB0AHQAZQByAEQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE4AZQB0AEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBOAGUAdABFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATgBlAHQARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEcAcgBvAHMAcwBFAG4AZQByAGcAeQBDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBHAHIAbwBzAHMARQBuAGUAcgBnAHkAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARwByAG8AcwBzAEUAbgBlAHIAZwB5AEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAZgBmAGkAYwBpAGUAbgBjAHkATwBmAFUAcwBlAE8AZgBNAGUAdABhAGIAbwBsAGkAegBhAGIAbABlAEUAbgBlAHIAZwB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAGYAZgBpAGMAaQBlAG4AYwB5AE8AZgBVAHMAZQBPAGYATQBlAHQAYQBiAG8AbABpAHoAYQBiAGwAZQBFAG4AZQByAGcAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBmAGYAaQBjAGkAZQBuAGMAeQBPAGYAVQBzAGUATwBmAE0AZQB0AGEAYgBvAGwAaQB6AGEAYgBsAGUARQBuAGUAcgBnAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAEYAbwByAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIARgBvAHIATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBGAG8AcgBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAGgAcgBvAHUAZwBoAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAaAByAG8AdQBnAGgATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABoAHIAbwB1AGcAaABMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8ARgBhAHQAQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBGAGEAdABDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAEYAYQB0AEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQBfAFAAcgBvAHQAZQBpAG4AQwBvAG4AdABlAG4AdABJAG4ATQBpAGwAawBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAGkAcgB5AF8AUAByAG8AdABlAGkAbgBDAG8AbgB0AGUAbgB0AEkAbgBNAGkAbABrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQBpAHIAeQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAaQByAHkAXwBQAHIAbwB0AGUAaQBuAEMAbwBuAHQAZQBuAHQASQBuAE0AaQBsAGsAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwAzAF8ARAByAHkATQBhAHQAdABlAHIARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8AMwBfAEQAcgB5AE0AYQB0AHQAZQByAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADMAXwBEAHIAeQBNAGEAdAB0AGUAcgBGAGUAZQBkAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANABfAEEAZABkAGkAdABpAG8AbgBhAGwASQBuAHQAYQBrAGUARgBvAHIATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA0AF8AQQBkAGQAaQB0AGkAbwBuAGEAbABJAG4AdABhAGsAZQBGAG8AcgBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADQAXwBBAGQAZABpAHQAaQBvAG4AYQBsAEkAbgB0AGEAawBlAEYAbwByAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADUAXwBNAGkAbABrAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGkAbABrAFMAbwBsAGkAZABzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANQBfAE0AaQBsAGsAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AaQBsAGsAUwBvAGwAaQBkAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA1AF8ATQBpAGwAawBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBpAGwAawBTAG8AbABpAGQAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEQAYQBpAHIAeQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADMAXwAxAF8AMQBfAF8ANgBfAE0AZQB0AGEAYgBvAGwAaQBzAGEAYgBpAGwAaQB0AHkATwBmAEQAaQBlAHQAXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBEAGEAaQByAHkAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAzAF8AMQBfADEAXwBfADYAXwBNAGUAdABhAGIAbwBsAGkAcwBhAGIAaQBsAGkAdAB5AE8AZgBEAGkAZQB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARABhAGkAcgB5AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMwBfADEAXwAxAF8AXwA2AF8ATQBlAHQAYQBiAG8AbABpAHMAYQBiAGkAbABpAHQAeQBPAGYARABpAGUAdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4ATQBNAFMAQQBmAHQAZQByAFMAbwBsAGkAZABTAGUAcABhAHIAYQB0AGkAbwBuACIALAAiAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwBfAEQAYQBpAHIAeQAuAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgBdACwAIgBsAG8AYwBhAGwAZQAiADoAewAiAGwAaQBzAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgByAG8AdwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGMAbwBsAHUAbQBuAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBQAG8AcwBpAHQAaQBvAG4AcwAiADoAWwAzAF0ALAAiAGQAZQBjAGkAbQBhAGwAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALgAiACwAIgBkAGEAdABlAE8AcgBkAGUAcgAiADoAIgBEAE0AWQAiACwAIgBjAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwAIgA6ACIAJAAiACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsAEwAZQBhAGQAIgA6AHQAcgB1AGUALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwBlAHAAQgB5AFMAcABhAGMAZQAiADoAZgBhAGwAcwBlACwAIgByAG8AdwBMAGUAdAB0AGUAcgAiADoAIgBSACIALAAiAGMAbwBsAHUAbQBuAEwAZQB0AHQAZQByACIAOgAiAEMAIgAsACIAcgBjAEwAZQBmAHQAQgByAGEAYwBrAGUAdAAiADoAIgBbACIALAAiAHIAYwBSAGkAZwBoAHQAQgByAGEAYwBrAGUAdAAiADoAIgBdACIALAAiAHMAdABhAHQAZQBtAGUAbgB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAbABvAGMAYQBsAGUATgBhAG0AZQAiADoAIgBlAG4ALQB1AHMAIgB9AH0A</AFEJSONBlob>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -25870,12 +25817,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -25889,9 +25833,12 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>